<commit_message>
feat(battle): add participant and card pile HUD
</commit_message>
<xml_diff>
--- a/DataTables/Datas/i18n.xlsx
+++ b/DataTables/Datas/i18n.xlsx
@@ -61,7 +61,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -319,12 +319,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Test Warrior</t>
+          <t>Sisyphus</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>测试战士</t>
+          <t>西西弗斯</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -341,12 +341,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Test Slime</t>
+          <t>Warden</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>测试史莱姆</t>
+          <t>典狱长</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -355,7 +355,73 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>battle.card_pile.draw.name</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Draw Pile</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>抽牌堆</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>battle.card_pile.discard.name</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Discard Pile</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>弃牌堆</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>battle.card_pile.exhaust.name</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Exhaust Pile</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>消耗牌堆</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D11"/>
+  <autoFilter ref="A1:D16"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(run): add G1-A entry and first-battle lifecycle
</commit_message>
<xml_diff>
--- a/DataTables/Datas/i18n.xlsx
+++ b/DataTables/Datas/i18n.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="i18n" sheetId="1" r:id="R06484a7c327c4be9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="i18n" sheetId="1" r:id="R7dad5c5acdcc4715"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -487,10 +487,10 @@
         <x:v>battle.hero.test_warrior.name</x:v>
       </x:c>
       <x:c r="B12" s="7" t="str">
-        <x:v>Sisyphus</x:v>
+        <x:v>Warrior</x:v>
       </x:c>
       <x:c r="C12" s="8" t="str">
-        <x:v>西西弗斯</x:v>
+        <x:v>战士</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
         <x:v>false</x:v>
@@ -7606,6 +7606,258 @@
       </x:c>
       <x:c r="D520" t="str">
         <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="521">
+      <x:c r="A521" t="str">
+        <x:v>run.entry.title</x:v>
+      </x:c>
+      <x:c r="B521" t="str">
+        <x:v>TinySpire</x:v>
+      </x:c>
+      <x:c r="C521" t="str">
+        <x:v>TinySpire</x:v>
+      </x:c>
+      <x:c r="D521" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="522">
+      <x:c r="A522" t="str">
+        <x:v>run.entry.menu.start</x:v>
+      </x:c>
+      <x:c r="B522" t="str">
+        <x:v>Start Game</x:v>
+      </x:c>
+      <x:c r="C522" t="str">
+        <x:v>开始游戏</x:v>
+      </x:c>
+      <x:c r="D522" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="523">
+      <x:c r="A523" t="str">
+        <x:v>run.entry.menu.settings</x:v>
+      </x:c>
+      <x:c r="B523" t="str">
+        <x:v>Settings</x:v>
+      </x:c>
+      <x:c r="C523" t="str">
+        <x:v>设置</x:v>
+      </x:c>
+      <x:c r="D523" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="524">
+      <x:c r="A524" t="str">
+        <x:v>run.entry.menu.compendium</x:v>
+      </x:c>
+      <x:c r="B524" t="str">
+        <x:v>Compendium</x:v>
+      </x:c>
+      <x:c r="C524" t="str">
+        <x:v>图鉴</x:v>
+      </x:c>
+      <x:c r="D524" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="525">
+      <x:c r="A525" t="str">
+        <x:v>run.entry.menu.statistics</x:v>
+      </x:c>
+      <x:c r="B525" t="str">
+        <x:v>Statistics</x:v>
+      </x:c>
+      <x:c r="C525" t="str">
+        <x:v>统计</x:v>
+      </x:c>
+      <x:c r="D525" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="526">
+      <x:c r="A526" t="str">
+        <x:v>run.entry.common.back</x:v>
+      </x:c>
+      <x:c r="B526" t="str">
+        <x:v>Back</x:v>
+      </x:c>
+      <x:c r="C526" t="str">
+        <x:v>返回</x:v>
+      </x:c>
+      <x:c r="D526" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="527">
+      <x:c r="A527" t="str">
+        <x:v>run.entry.common.coming_soon</x:v>
+      </x:c>
+      <x:c r="B527" t="str">
+        <x:v>In Development</x:v>
+      </x:c>
+      <x:c r="C527" t="str">
+        <x:v>开发中</x:v>
+      </x:c>
+      <x:c r="D527" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="528">
+      <x:c r="A528" t="str">
+        <x:v>run.entry.settings.title</x:v>
+      </x:c>
+      <x:c r="B528" t="str">
+        <x:v>Settings</x:v>
+      </x:c>
+      <x:c r="C528" t="str">
+        <x:v>设置</x:v>
+      </x:c>
+      <x:c r="D528" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="529">
+      <x:c r="A529" t="str">
+        <x:v>run.entry.settings.placeholder</x:v>
+      </x:c>
+      <x:c r="B529" t="str">
+        <x:v>Settings layout placeholder</x:v>
+      </x:c>
+      <x:c r="C529" t="str">
+        <x:v>设置布局占位</x:v>
+      </x:c>
+      <x:c r="D529" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="530">
+      <x:c r="A530" t="str">
+        <x:v>run.entry.hero.title</x:v>
+      </x:c>
+      <x:c r="B530" t="str">
+        <x:v>Choose a Hero</x:v>
+      </x:c>
+      <x:c r="C530" t="str">
+        <x:v>选择角色</x:v>
+      </x:c>
+      <x:c r="D530" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="531">
+      <x:c r="A531" t="str">
+        <x:v>run.entry.hero.confirm</x:v>
+      </x:c>
+      <x:c r="B531" t="str">
+        <x:v>Start Run</x:v>
+      </x:c>
+      <x:c r="C531" t="str">
+        <x:v>确认并开始</x:v>
+      </x:c>
+      <x:c r="D531" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="532">
+      <x:c r="A532" t="str">
+        <x:v>run.entry.hero.future_slot</x:v>
+      </x:c>
+      <x:c r="B532" t="str">
+        <x:v>Future Team Slot</x:v>
+      </x:c>
+      <x:c r="C532" t="str">
+        <x:v>未来队伍槽位</x:v>
+      </x:c>
+      <x:c r="D532" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="533">
+      <x:c r="A533" t="str">
+        <x:v>run.entry.map.title</x:v>
+      </x:c>
+      <x:c r="B533" t="str">
+        <x:v>Temporary Map</x:v>
+      </x:c>
+      <x:c r="C533" t="str">
+        <x:v>临时地图</x:v>
+      </x:c>
+      <x:c r="D533" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="534">
+      <x:c r="A534" t="str">
+        <x:v>run.entry.map.battle_node</x:v>
+      </x:c>
+      <x:c r="B534" t="str">
+        <x:v>First Battle</x:v>
+      </x:c>
+      <x:c r="C534" t="str">
+        <x:v>首战</x:v>
+      </x:c>
+      <x:c r="D534" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="535">
+      <x:c r="A535" t="str">
+        <x:v>run.entry.map.cleared</x:v>
+      </x:c>
+      <x:c r="B535" t="str">
+        <x:v>Cleared</x:v>
+      </x:c>
+      <x:c r="C535" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="D535" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="536">
+      <x:c r="A536" t="str">
+        <x:v>run.entry.map.health</x:v>
+      </x:c>
+      <x:c r="B536" t="str">
+        <x:v>HP {current}/{max}</x:v>
+      </x:c>
+      <x:c r="C536" t="str">
+        <x:v>生命 {current}/{max}</x:v>
+      </x:c>
+      <x:c r="D536" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="537">
+      <x:c r="A537" t="str">
+        <x:v>run.entry.failure.title</x:v>
+      </x:c>
+      <x:c r="B537" t="str">
+        <x:v>Battle Failed</x:v>
+      </x:c>
+      <x:c r="C537" t="str">
+        <x:v>战斗失败</x:v>
+      </x:c>
+      <x:c r="D537" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="538">
+      <x:c r="A538" t="str">
+        <x:v>run.entry.failure.restart</x:v>
+      </x:c>
+      <x:c r="B538" t="str">
+        <x:v>Restart Battle</x:v>
+      </x:c>
+      <x:c r="C538" t="str">
+        <x:v>重开本关</x:v>
+      </x:c>
+      <x:c r="D538" t="str">
+        <x:v>false</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(run): add G2-A persistence and continue flow
</commit_message>
<xml_diff>
--- a/DataTables/Datas/i18n.xlsx
+++ b/DataTables/Datas/i18n.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="i18n" sheetId="1" r:id="R7dad5c5acdcc4715"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="i18n" sheetId="1" r:id="R81e92ce9428e4bf4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7809,10 +7809,10 @@
         <x:v>run.entry.map.cleared</x:v>
       </x:c>
       <x:c r="B535" t="str">
-        <x:v>Cleared</x:v>
+        <x:v>Node cleared; later content is not connected yet</x:v>
       </x:c>
       <x:c r="C535" t="str">
-        <x:v>已完成</x:v>
+        <x:v>节点已清除、后续内容未接入</x:v>
       </x:c>
       <x:c r="D535" t="str">
         <x:v>false</x:v>
@@ -7857,6 +7857,314 @@
         <x:v>重开本关</x:v>
       </x:c>
       <x:c r="D538" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="539">
+      <x:c r="A539" t="str">
+        <x:v>run.entry.menu.continue</x:v>
+      </x:c>
+      <x:c r="B539" t="str">
+        <x:v>Continue</x:v>
+      </x:c>
+      <x:c r="C539" t="str">
+        <x:v>继续游戏</x:v>
+      </x:c>
+      <x:c r="D539" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="540">
+      <x:c r="A540" t="str">
+        <x:v>run.entry.common.cancel</x:v>
+      </x:c>
+      <x:c r="B540" t="str">
+        <x:v>Cancel</x:v>
+      </x:c>
+      <x:c r="C540" t="str">
+        <x:v>取消</x:v>
+      </x:c>
+      <x:c r="D540" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="541">
+      <x:c r="A541" t="str">
+        <x:v>run.entry.abandon.title</x:v>
+      </x:c>
+      <x:c r="B541" t="str">
+        <x:v>Abandon current Run?</x:v>
+      </x:c>
+      <x:c r="C541" t="str">
+        <x:v>放弃当前 Run？</x:v>
+      </x:c>
+      <x:c r="D541" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="542">
+      <x:c r="A542" t="str">
+        <x:v>run.entry.abandon.message</x:v>
+      </x:c>
+      <x:c r="B542" t="str">
+        <x:v>The current save will be deleted before starting a new Run.</x:v>
+      </x:c>
+      <x:c r="C542" t="str">
+        <x:v>开始新 Run 前会删除当前存档。</x:v>
+      </x:c>
+      <x:c r="D542" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="543">
+      <x:c r="A543" t="str">
+        <x:v>run.entry.abandon.confirm</x:v>
+      </x:c>
+      <x:c r="B543" t="str">
+        <x:v>Abandon Run</x:v>
+      </x:c>
+      <x:c r="C543" t="str">
+        <x:v>放弃 Run</x:v>
+      </x:c>
+      <x:c r="D543" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="544">
+      <x:c r="A544" t="str">
+        <x:v>run.entry.save.issue.title</x:v>
+      </x:c>
+      <x:c r="B544" t="str">
+        <x:v>Save Unavailable</x:v>
+      </x:c>
+      <x:c r="C544" t="str">
+        <x:v>存档不可用</x:v>
+      </x:c>
+      <x:c r="D544" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="545">
+      <x:c r="A545" t="str">
+        <x:v>run.entry.save.issue.invalid_json</x:v>
+      </x:c>
+      <x:c r="B545" t="str">
+        <x:v>The save file contains invalid JSON. Continue is unavailable.</x:v>
+      </x:c>
+      <x:c r="C545" t="str">
+        <x:v>存档不是有效的 JSON，无法继续游戏。</x:v>
+      </x:c>
+      <x:c r="D545" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="546">
+      <x:c r="A546" t="str">
+        <x:v>run.entry.save.issue.invalid_document</x:v>
+      </x:c>
+      <x:c r="B546" t="str">
+        <x:v>The save data is incomplete or invalid. Continue is unavailable.</x:v>
+      </x:c>
+      <x:c r="C546" t="str">
+        <x:v>存档内容不完整或无效，无法继续游戏。</x:v>
+      </x:c>
+      <x:c r="D546" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="547">
+      <x:c r="A547" t="str">
+        <x:v>run.entry.save.issue.unsupported_schema</x:v>
+      </x:c>
+      <x:c r="B547" t="str">
+        <x:v>This save version is unknown or cannot be migrated. Continue is unavailable.</x:v>
+      </x:c>
+      <x:c r="C547" t="str">
+        <x:v>存档版本未知或无法迁移，无法继续游戏。</x:v>
+      </x:c>
+      <x:c r="D547" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="548">
+      <x:c r="A548" t="str">
+        <x:v>run.entry.save.issue.interrupted_commit</x:v>
+      </x:c>
+      <x:c r="B548" t="str">
+        <x:v>An interrupted save was detected. Continue is unavailable.</x:v>
+      </x:c>
+      <x:c r="C548" t="str">
+        <x:v>检测到未完成的存档写入，无法继续游戏。</x:v>
+      </x:c>
+      <x:c r="D548" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="549">
+      <x:c r="A549" t="str">
+        <x:v>run.entry.save.issue.io_failure</x:v>
+      </x:c>
+      <x:c r="B549" t="str">
+        <x:v>The save could not be read. Continue is unavailable.</x:v>
+      </x:c>
+      <x:c r="C549" t="str">
+        <x:v>无法读取存档，无法继续游戏。</x:v>
+      </x:c>
+      <x:c r="D549" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="550">
+      <x:c r="A550" t="str">
+        <x:v>run.entry.save.issue.missing_configuration</x:v>
+      </x:c>
+      <x:c r="B550" t="str">
+        <x:v>The save references missing {kind} configuration ID {id}. Continue is unavailable.</x:v>
+      </x:c>
+      <x:c r="C550" t="str">
+        <x:v>存档引用的 {kind} 配置 ID {id} 缺失，无法继续游戏。</x:v>
+      </x:c>
+      <x:c r="D550" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="551">
+      <x:c r="A551" t="str">
+        <x:v>run.entry.save.delete.title</x:v>
+      </x:c>
+      <x:c r="B551" t="str">
+        <x:v>Delete unusable save?</x:v>
+      </x:c>
+      <x:c r="C551" t="str">
+        <x:v>删除不可用的存档？</x:v>
+      </x:c>
+      <x:c r="D551" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="552">
+      <x:c r="A552" t="str">
+        <x:v>run.entry.save.delete.message</x:v>
+      </x:c>
+      <x:c r="B552" t="str">
+        <x:v>This save will be permanently deleted. This cannot be undone.</x:v>
+      </x:c>
+      <x:c r="C552" t="str">
+        <x:v>该存档将被永久删除，且无法撤销。</x:v>
+      </x:c>
+      <x:c r="D552" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="553">
+      <x:c r="A553" t="str">
+        <x:v>run.entry.save.delete.confirm</x:v>
+      </x:c>
+      <x:c r="B553" t="str">
+        <x:v>Delete Save</x:v>
+      </x:c>
+      <x:c r="C553" t="str">
+        <x:v>删除存档</x:v>
+      </x:c>
+      <x:c r="D553" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="554">
+      <x:c r="A554" t="str">
+        <x:v>run.entry.save.delete.failed</x:v>
+      </x:c>
+      <x:c r="B554" t="str">
+        <x:v>The save could not be deleted. Retry or cancel.</x:v>
+      </x:c>
+      <x:c r="C554" t="str">
+        <x:v>删除存档失败，请重试或取消。</x:v>
+      </x:c>
+      <x:c r="D554" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="555">
+      <x:c r="A555" t="str">
+        <x:v>run.entry.save.commit_failed</x:v>
+      </x:c>
+      <x:c r="B555" t="str">
+        <x:v>Save failed. Retry.</x:v>
+      </x:c>
+      <x:c r="C555" t="str">
+        <x:v>保存失败，请重试。</x:v>
+      </x:c>
+      <x:c r="D555" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="556">
+      <x:c r="A556" t="str">
+        <x:v>run.entry.save.retry</x:v>
+      </x:c>
+      <x:c r="B556" t="str">
+        <x:v>Retry Save</x:v>
+      </x:c>
+      <x:c r="C556" t="str">
+        <x:v>重试保存</x:v>
+      </x:c>
+      <x:c r="D556" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="557">
+      <x:c r="A557" t="str">
+        <x:v>run.entry.save.exit</x:v>
+      </x:c>
+      <x:c r="B557" t="str">
+        <x:v>Exit</x:v>
+      </x:c>
+      <x:c r="C557" t="str">
+        <x:v>退出</x:v>
+      </x:c>
+      <x:c r="D557" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="558">
+      <x:c r="A558" t="str">
+        <x:v>run.entry.save.rollback.title</x:v>
+      </x:c>
+      <x:c r="B558" t="str">
+        <x:v>Exit without saving?</x:v>
+      </x:c>
+      <x:c r="C558" t="str">
+        <x:v>不保存并退出？</x:v>
+      </x:c>
+      <x:c r="D558" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="559">
+      <x:c r="A559" t="str">
+        <x:v>run.entry.save.rollback.message</x:v>
+      </x:c>
+      <x:c r="B559" t="str">
+        <x:v>If you exit now, Continue will return to the last successfully saved map checkpoint. If no checkpoint was saved, this Run cannot be recovered.</x:v>
+      </x:c>
+      <x:c r="C559" t="str">
+        <x:v>现在退出后，“继续游戏”会回退到上一份成功保存的地图检查点；若尚无检查点，本 Run 将无法恢复。</x:v>
+      </x:c>
+      <x:c r="D559" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="560">
+      <x:c r="A560" t="str">
+        <x:v>run.entry.save.rollback.confirm</x:v>
+      </x:c>
+      <x:c r="B560" t="str">
+        <x:v>Exit and Roll Back</x:v>
+      </x:c>
+      <x:c r="C560" t="str">
+        <x:v>退出并回退</x:v>
+      </x:c>
+      <x:c r="D560" t="str">
         <x:v>false</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(run): add deterministic act map
</commit_message>
<xml_diff>
--- a/DataTables/Datas/i18n.xlsx
+++ b/DataTables/Datas/i18n.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="i18n" sheetId="1" r:id="R81e92ce9428e4bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="i18n" sheetId="1" r:id="Race14556d1714da0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7781,10 +7781,10 @@
         <x:v>run.entry.map.title</x:v>
       </x:c>
       <x:c r="B533" t="str">
-        <x:v>Temporary Map</x:v>
+        <x:v>Act Map</x:v>
       </x:c>
       <x:c r="C533" t="str">
-        <x:v>临时地图</x:v>
+        <x:v>Act 地图</x:v>
       </x:c>
       <x:c r="D533" t="str">
         <x:v>false</x:v>
@@ -7795,10 +7795,10 @@
         <x:v>run.entry.map.battle_node</x:v>
       </x:c>
       <x:c r="B534" t="str">
-        <x:v>First Battle</x:v>
+        <x:v>Encounter</x:v>
       </x:c>
       <x:c r="C534" t="str">
-        <x:v>首战</x:v>
+        <x:v>遭遇</x:v>
       </x:c>
       <x:c r="D534" t="str">
         <x:v>false</x:v>

</xml_diff>

<commit_message>
feat(run): complete G8 productization gates
</commit_message>
<xml_diff>
--- a/DataTables/Datas/i18n.xlsx
+++ b/DataTables/Datas/i18n.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="i18n" sheetId="1" r:id="R2c03c3113e60440f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="i18n" sheetId="1" r:id="R16bf0b8129b84eca"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -30,7 +30,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -62,6 +62,26 @@
         <x:fgColor rgb="FFE4DFEC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4DFEC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -69,7 +89,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="23">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -102,6 +122,26 @@
           <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
         </x:ext>
       </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -8644,6 +8684,566 @@
         <x:v>false</x:v>
       </x:c>
     </x:row>
+    <x:row r="595">
+      <x:c r="A595" s="13" t="str">
+        <x:v>app.settings.title</x:v>
+      </x:c>
+      <x:c r="B595" s="16" t="str">
+        <x:v>Settings</x:v>
+      </x:c>
+      <x:c r="C595" s="19" t="str">
+        <x:v>设置</x:v>
+      </x:c>
+      <x:c r="D595" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="596">
+      <x:c r="A596" s="13" t="str">
+        <x:v>app.settings.language</x:v>
+      </x:c>
+      <x:c r="B596" s="16" t="str">
+        <x:v>Language</x:v>
+      </x:c>
+      <x:c r="C596" s="19" t="str">
+        <x:v>语言</x:v>
+      </x:c>
+      <x:c r="D596" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="597">
+      <x:c r="A597" s="13" t="str">
+        <x:v>app.settings.language.en</x:v>
+      </x:c>
+      <x:c r="B597" s="16" t="str">
+        <x:v>English</x:v>
+      </x:c>
+      <x:c r="C597" s="19" t="str">
+        <x:v>English</x:v>
+      </x:c>
+      <x:c r="D597" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="598">
+      <x:c r="A598" s="13" t="str">
+        <x:v>app.settings.language.zh_cn</x:v>
+      </x:c>
+      <x:c r="B598" s="16" t="str">
+        <x:v>Simplified Chinese</x:v>
+      </x:c>
+      <x:c r="C598" s="19" t="str">
+        <x:v>简体中文</x:v>
+      </x:c>
+      <x:c r="D598" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="599">
+      <x:c r="A599" s="13" t="str">
+        <x:v>app.settings.master_volume</x:v>
+      </x:c>
+      <x:c r="B599" s="16" t="str">
+        <x:v>Master Volume</x:v>
+      </x:c>
+      <x:c r="C599" s="19" t="str">
+        <x:v>主音量</x:v>
+      </x:c>
+      <x:c r="D599" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="600">
+      <x:c r="A600" s="13" t="str">
+        <x:v>app.settings.display_mode</x:v>
+      </x:c>
+      <x:c r="B600" s="16" t="str">
+        <x:v>Display Mode</x:v>
+      </x:c>
+      <x:c r="C600" s="19" t="str">
+        <x:v>显示模式</x:v>
+      </x:c>
+      <x:c r="D600" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="601">
+      <x:c r="A601" s="13" t="str">
+        <x:v>app.settings.display_mode.windowed</x:v>
+      </x:c>
+      <x:c r="B601" s="16" t="str">
+        <x:v>Windowed</x:v>
+      </x:c>
+      <x:c r="C601" s="19" t="str">
+        <x:v>窗口化</x:v>
+      </x:c>
+      <x:c r="D601" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="602">
+      <x:c r="A602" s="13" t="str">
+        <x:v>app.settings.display_mode.borderless</x:v>
+      </x:c>
+      <x:c r="B602" s="16" t="str">
+        <x:v>Borderless Fullscreen</x:v>
+      </x:c>
+      <x:c r="C602" s="19" t="str">
+        <x:v>无边框全屏</x:v>
+      </x:c>
+      <x:c r="D602" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="603">
+      <x:c r="A603" s="13" t="str">
+        <x:v>app.settings.resolution</x:v>
+      </x:c>
+      <x:c r="B603" s="16" t="str">
+        <x:v>Resolution</x:v>
+      </x:c>
+      <x:c r="C603" s="19" t="str">
+        <x:v>分辨率</x:v>
+      </x:c>
+      <x:c r="D603" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="604">
+      <x:c r="A604" s="13" t="str">
+        <x:v>app.settings.text_scale</x:v>
+      </x:c>
+      <x:c r="B604" s="16" t="str">
+        <x:v>Text Scale</x:v>
+      </x:c>
+      <x:c r="C604" s="19" t="str">
+        <x:v>文字缩放</x:v>
+      </x:c>
+      <x:c r="D604" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="605">
+      <x:c r="A605" s="13" t="str">
+        <x:v>app.settings.high_contrast</x:v>
+      </x:c>
+      <x:c r="B605" s="16" t="str">
+        <x:v>High Contrast</x:v>
+      </x:c>
+      <x:c r="C605" s="19" t="str">
+        <x:v>高对比度</x:v>
+      </x:c>
+      <x:c r="D605" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="606">
+      <x:c r="A606" s="13" t="str">
+        <x:v>app.settings.reduced_motion</x:v>
+      </x:c>
+      <x:c r="B606" s="16" t="str">
+        <x:v>Reduced Motion</x:v>
+      </x:c>
+      <x:c r="C606" s="19" t="str">
+        <x:v>减少动态效果</x:v>
+      </x:c>
+      <x:c r="D606" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="607">
+      <x:c r="A607" s="13" t="str">
+        <x:v>app.settings.state.enabled</x:v>
+      </x:c>
+      <x:c r="B607" s="16" t="str">
+        <x:v>Enabled</x:v>
+      </x:c>
+      <x:c r="C607" s="19" t="str">
+        <x:v>已启用</x:v>
+      </x:c>
+      <x:c r="D607" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="608">
+      <x:c r="A608" s="13" t="str">
+        <x:v>app.settings.state.disabled</x:v>
+      </x:c>
+      <x:c r="B608" s="16" t="str">
+        <x:v>Disabled</x:v>
+      </x:c>
+      <x:c r="C608" s="19" t="str">
+        <x:v>已关闭</x:v>
+      </x:c>
+      <x:c r="D608" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="609">
+      <x:c r="A609" s="13" t="str">
+        <x:v>app.settings.action.decrease</x:v>
+      </x:c>
+      <x:c r="B609" s="16" t="str">
+        <x:v>Decrease</x:v>
+      </x:c>
+      <x:c r="C609" s="19" t="str">
+        <x:v>降低</x:v>
+      </x:c>
+      <x:c r="D609" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="610">
+      <x:c r="A610" s="13" t="str">
+        <x:v>app.settings.action.increase</x:v>
+      </x:c>
+      <x:c r="B610" s="16" t="str">
+        <x:v>Increase</x:v>
+      </x:c>
+      <x:c r="C610" s="19" t="str">
+        <x:v>提高</x:v>
+      </x:c>
+      <x:c r="D610" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="611">
+      <x:c r="A611" s="13" t="str">
+        <x:v>app.settings.action.previous</x:v>
+      </x:c>
+      <x:c r="B611" s="16" t="str">
+        <x:v>Previous</x:v>
+      </x:c>
+      <x:c r="C611" s="19" t="str">
+        <x:v>上一个</x:v>
+      </x:c>
+      <x:c r="D611" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="612">
+      <x:c r="A612" s="13" t="str">
+        <x:v>app.settings.action.next</x:v>
+      </x:c>
+      <x:c r="B612" s="16" t="str">
+        <x:v>Next</x:v>
+      </x:c>
+      <x:c r="C612" s="19" t="str">
+        <x:v>下一个</x:v>
+      </x:c>
+      <x:c r="D612" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="613">
+      <x:c r="A613" s="13" t="str">
+        <x:v>app.settings.failure.save</x:v>
+      </x:c>
+      <x:c r="B613" s="16" t="str">
+        <x:v>Settings could not be saved. The previous values are still active.</x:v>
+      </x:c>
+      <x:c r="C613" s="19" t="str">
+        <x:v>设置无法保存，当前仍使用修改前的值。</x:v>
+      </x:c>
+      <x:c r="D613" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="614">
+      <x:c r="A614" s="13" t="str">
+        <x:v>app.settings.failure.unsupported_resolution</x:v>
+      </x:c>
+      <x:c r="B614" s="16" t="str">
+        <x:v>This resolution is not in the supported release matrix.</x:v>
+      </x:c>
+      <x:c r="C614" s="19" t="str">
+        <x:v>该分辨率不在本次发布支持矩阵中。</x:v>
+      </x:c>
+      <x:c r="D614" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="615">
+      <x:c r="A615" s="13" t="str">
+        <x:v>tutorial.guide.main_menu_welcome</x:v>
+      </x:c>
+      <x:c r="B615" s="16" t="str">
+        <x:v>Welcome. Start a Run, choose a hero, then climb one connected route through the Act.</x:v>
+      </x:c>
+      <x:c r="C615" s="19" t="str">
+        <x:v>欢迎。开始一局游戏，选择英雄，然后沿连通路线完成这一幕。</x:v>
+      </x:c>
+      <x:c r="D615" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="616">
+      <x:c r="A616" s="13" t="str">
+        <x:v>tutorial.guide.hero_selection</x:v>
+      </x:c>
+      <x:c r="B616" s="16" t="str">
+        <x:v>Choose a hero to lock the starting deck and Run identity.</x:v>
+      </x:c>
+      <x:c r="C616" s="19" t="str">
+        <x:v>选择英雄后，将确定初始牌组和本局身份。</x:v>
+      </x:c>
+      <x:c r="D616" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="617">
+      <x:c r="A617" s="13" t="str">
+        <x:v>tutorial.guide.map_route</x:v>
+      </x:c>
+      <x:c r="B617" s="16" t="str">
+        <x:v>Choose any reachable node. Cleared nodes stay cleared, and only connected routes unlock.</x:v>
+      </x:c>
+      <x:c r="C617" s="19" t="str">
+        <x:v>请选择可到达的节点。已完成节点会保留，只有相连路线会解锁。</x:v>
+      </x:c>
+      <x:c r="D617" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="618">
+      <x:c r="A618" s="13" t="str">
+        <x:v>tutorial.guide.battle_basics</x:v>
+      </x:c>
+      <x:c r="B618" s="16" t="str">
+        <x:v>Drag a card onto a valid target, watch energy and intent, then end the turn when ready.</x:v>
+      </x:c>
+      <x:c r="C618" s="19" t="str">
+        <x:v>将卡牌拖到有效目标，留意能量和敌人意图，准备好后结束回合。</x:v>
+      </x:c>
+      <x:c r="D618" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="619">
+      <x:c r="A619" s="13" t="str">
+        <x:v>tutorial.guide.card_reward</x:v>
+      </x:c>
+      <x:c r="B619" s="16" t="str">
+        <x:v>After battle, take one reward card or skip it. Your choice is saved immediately.</x:v>
+      </x:c>
+      <x:c r="C619" s="19" t="str">
+        <x:v>战斗后可选择一张奖励卡，或跳过奖励。选择会立即保存。</x:v>
+      </x:c>
+      <x:c r="D619" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="620">
+      <x:c r="A620" s="13" t="str">
+        <x:v>tutorial.guide.non_combat_node</x:v>
+      </x:c>
+      <x:c r="B620" s="16" t="str">
+        <x:v>Rest, chest, shop, and event nodes resolve once. Review the choice before confirming.</x:v>
+      </x:c>
+      <x:c r="C620" s="19" t="str">
+        <x:v>休息、宝箱、商店和事件节点只结算一次，请在确认前检查选择。</x:v>
+      </x:c>
+      <x:c r="D620" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="621">
+      <x:c r="A621" s="13" t="str">
+        <x:v>tutorial.guide.run_outcome</x:v>
+      </x:c>
+      <x:c r="B621" s="16" t="str">
+        <x:v>The Run is over. Review the result, then return to the menu; the summary remains in Statistics.</x:v>
+      </x:c>
+      <x:c r="C621" s="19" t="str">
+        <x:v>本局已经结束。查看结算后返回菜单，摘要会保留在统计记录中。</x:v>
+      </x:c>
+      <x:c r="D621" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="622">
+      <x:c r="A622" s="13" t="str">
+        <x:v>tutorial.guide.confirm</x:v>
+      </x:c>
+      <x:c r="B622" s="16" t="str">
+        <x:v>Got it</x:v>
+      </x:c>
+      <x:c r="C622" s="19" t="str">
+        <x:v>知道了</x:v>
+      </x:c>
+      <x:c r="D622" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="623">
+      <x:c r="A623" s="13" t="str">
+        <x:v>tutorial.guide.skip</x:v>
+      </x:c>
+      <x:c r="B623" s="16" t="str">
+        <x:v>Skip tutorial</x:v>
+      </x:c>
+      <x:c r="C623" s="19" t="str">
+        <x:v>跳过教程</x:v>
+      </x:c>
+      <x:c r="D623" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="624">
+      <x:c r="A624" s="13" t="str">
+        <x:v>tutorial.guide.reset</x:v>
+      </x:c>
+      <x:c r="B624" s="16" t="str">
+        <x:v>Reset tutorial</x:v>
+      </x:c>
+      <x:c r="C624" s="19" t="str">
+        <x:v>重置教程</x:v>
+      </x:c>
+      <x:c r="D624" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="625">
+      <x:c r="A625" s="13" t="str">
+        <x:v>app.statistics.title</x:v>
+      </x:c>
+      <x:c r="B625" s="16" t="str">
+        <x:v>Run Statistics</x:v>
+      </x:c>
+      <x:c r="C625" s="19" t="str">
+        <x:v>游戏统计</x:v>
+      </x:c>
+      <x:c r="D625" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="626">
+      <x:c r="A626" s="13" t="str">
+        <x:v>app.statistics.total_runs</x:v>
+      </x:c>
+      <x:c r="B626" s="16" t="str">
+        <x:v>Total Runs</x:v>
+      </x:c>
+      <x:c r="C626" s="19" t="str">
+        <x:v>总局数</x:v>
+      </x:c>
+      <x:c r="D626" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="627">
+      <x:c r="A627" s="13" t="str">
+        <x:v>app.statistics.victory</x:v>
+      </x:c>
+      <x:c r="B627" s="16" t="str">
+        <x:v>Victories</x:v>
+      </x:c>
+      <x:c r="C627" s="19" t="str">
+        <x:v>胜利</x:v>
+      </x:c>
+      <x:c r="D627" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="628">
+      <x:c r="A628" s="13" t="str">
+        <x:v>app.statistics.defeat</x:v>
+      </x:c>
+      <x:c r="B628" s="16" t="str">
+        <x:v>Defeats</x:v>
+      </x:c>
+      <x:c r="C628" s="19" t="str">
+        <x:v>失败</x:v>
+      </x:c>
+      <x:c r="D628" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="629">
+      <x:c r="A629" s="13" t="str">
+        <x:v>app.statistics.abandoned</x:v>
+      </x:c>
+      <x:c r="B629" s="16" t="str">
+        <x:v>Abandoned</x:v>
+      </x:c>
+      <x:c r="C629" s="19" t="str">
+        <x:v>主动放弃</x:v>
+      </x:c>
+      <x:c r="D629" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="630">
+      <x:c r="A630" s="13" t="str">
+        <x:v>app.statistics.victory_rate</x:v>
+      </x:c>
+      <x:c r="B630" s="16" t="str">
+        <x:v>Victory Rate</x:v>
+      </x:c>
+      <x:c r="C630" s="19" t="str">
+        <x:v>胜率</x:v>
+      </x:c>
+      <x:c r="D630" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="631">
+      <x:c r="A631" s="13" t="str">
+        <x:v>app.statistics.hero</x:v>
+      </x:c>
+      <x:c r="B631" s="16" t="str">
+        <x:v>Hero {hero_template_id}</x:v>
+      </x:c>
+      <x:c r="C631" s="19" t="str">
+        <x:v>英雄 {hero_template_id}</x:v>
+      </x:c>
+      <x:c r="D631" s="22" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="632">
+      <x:c r="A632" s="13" t="str">
+        <x:v>app.statistics.empty</x:v>
+      </x:c>
+      <x:c r="B632" s="16" t="str">
+        <x:v>No completed Runs yet.</x:v>
+      </x:c>
+      <x:c r="C632" s="19" t="str">
+        <x:v>还没有已结束的游戏记录。</x:v>
+      </x:c>
+      <x:c r="D632" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="633">
+      <x:c r="A633" s="13" t="str">
+        <x:v>app.statistics.failure.load</x:v>
+      </x:c>
+      <x:c r="B633" s="16" t="str">
+        <x:v>Run history is unavailable: {detail}</x:v>
+      </x:c>
+      <x:c r="C633" s="19" t="str">
+        <x:v>游戏记录暂时不可用：{detail}</x:v>
+      </x:c>
+      <x:c r="D633" s="22" t="str">
+        <x:v>true</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="634">
+      <x:c r="A634" s="13" t="str">
+        <x:v>run.history.failure.record</x:v>
+      </x:c>
+      <x:c r="B634" s="16" t="str">
+        <x:v>The Run summary could not be recorded. The terminal save was kept; try again before leaving.</x:v>
+      </x:c>
+      <x:c r="C634" s="19" t="str">
+        <x:v>本局摘要无法写入。终局存档已保留，请重试后再离开。</x:v>
+      </x:c>
+      <x:c r="D634" s="22" t="str">
+        <x:v>false</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>